<commit_message>
Removed /v1/search options and MLCP tasks, dependency, etc.  Documentation updates.
</commit_message>
<xml_diff>
--- a/docs/lux-markdown-tables.xlsx
+++ b/docs/lux-markdown-tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\yale\clones\lux-marklogic\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EA00D6D-A59B-4379-A824-68D03D0BAA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5CF745-D248-4CDD-BA38-8BE0A74DCE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>Path</t>
   </si>
@@ -58,9 +58,6 @@
     <t>[/ml-modules](/src/main/ml-modules)</t>
   </si>
   <si>
-    <t>/v1/search options, which this project does not use.</t>
-  </si>
-  <si>
     <t>A few utility functions and classes used by the library code.</t>
   </si>
   <si>
@@ -193,9 +190,6 @@
     <t>[/root](/src/main/ml-modules/root)</t>
   </si>
   <si>
-    <t>[/options](/src/main/ml-modules/options)</t>
-  </si>
-  <si>
     <t>The modules applicable to all environments.</t>
   </si>
   <si>
@@ -254,6 +248,18 @@
   </si>
   <si>
     <t>[MarkLogic Unit Test user guide](https://marklogic-community.github.io/marklogic-unit-test/)</t>
+  </si>
+  <si>
+    <t>[/dynamic-host](/src/main/ml-config/dynamic-host)</t>
+  </si>
+  <si>
+    <t>Include in all ML 12 deployments, even those that do not require scaling out.  Once we no longer support ML 11, we can merge these settings into the base ml-config dir.</t>
+  </si>
+  <si>
+    <t>[/oauth](/src/main/ml-config/oauth)</t>
+  </si>
+  <si>
+    <t>Tenants with the My Collections feature enabled need to switch from digest to OAuth.</t>
   </si>
 </sst>
 </file>
@@ -591,30 +597,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="65.53515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="57" customWidth="1"/>
-    <col min="7" max="7" width="85.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.53515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="85.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
@@ -623,18 +629,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -642,203 +648,211 @@
         <v>4</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
         <v>19</v>
       </c>
-      <c r="F4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
         <v>25</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
         <v>26</v>
       </c>
-      <c r="G8" t="s">
+      <c r="F9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E22" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="D10" t="s">
+      <c r="G24" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" t="s">
         <v>29</v>
       </c>
-      <c r="F10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="D11" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="C12" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="C13" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="D14" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="D15" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E16" t="s">
-        <v>57</v>
-      </c>
-      <c r="F16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E17" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E18" t="s">
-        <v>59</v>
-      </c>
-      <c r="F18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="G27" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E19" t="s">
-        <v>60</v>
-      </c>
-      <c r="F19" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E20" t="s">
-        <v>61</v>
-      </c>
-      <c r="F20" t="s">
-        <v>63</v>
-      </c>
-      <c r="G20" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E21" t="s">
-        <v>62</v>
-      </c>
-      <c r="F21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="C22" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="B23" t="s">
-        <v>69</v>
-      </c>
-      <c r="G23" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="C24" t="s">
-        <v>70</v>
-      </c>
-      <c r="F24" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="C25" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" t="s">
-        <v>74</v>
-      </c>
-      <c r="G25" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A26" t="s">
-        <v>16</v>
-      </c>
-      <c r="F26" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -850,75 +864,75 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44646EB7-BD93-4383-9A53-F145B54BA665}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.61328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="48.07421875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.23046875" style="1"/>
+    <col min="1" max="1" width="43.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="48.109375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.21875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="7" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="87.45" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="72.900000000000006" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#666: primary change is new dependence on the mlAuthentication build property.
</commit_message>
<xml_diff>
--- a/docs/lux-markdown-tables.xlsx
+++ b/docs/lux-markdown-tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\yale\clones\lux-marklogic\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\yale\clones\lux-marklogic-v3\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5CF745-D248-4CDD-BA38-8BE0A74DCE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CE8F3E-107D-4039-8CCC-3ADB654C5248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -259,7 +259,7 @@
     <t>[/oauth](/src/main/ml-config/oauth)</t>
   </si>
   <si>
-    <t>Tenants with the My Collections feature enabled need to switch from digest to OAuth.</t>
+    <t>Tenants with the My Collections feature enabled need to switch to OAuth.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
#666: global default setting for authentication scheme (#667)
* #666: primary change is new dependence on the mlAuthentication build property.

* #666: default config is for local/HTTP envs

* Set auth scheme based on protocol

Co-authored-by: Copilot <175728472+Copilot@users.noreply.github.com>

* Script to display OS settings we commonly check.

* Added more for processors and memory

* Added OS release info, a check for OS updates, and disk capacities & usage.

* Renamed

---------

Co-authored-by: brent-hartwig <brent.d.hartwig@gmail.com>
Co-authored-by: Copilot <175728472+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/lux-markdown-tables.xlsx
+++ b/docs/lux-markdown-tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\yale\clones\lux-marklogic\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\yale\clones\lux-marklogic-v3\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5CF745-D248-4CDD-BA38-8BE0A74DCE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CE8F3E-107D-4039-8CCC-3ADB654C5248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -259,7 +259,7 @@
     <t>[/oauth](/src/main/ml-config/oauth)</t>
   </si>
   <si>
-    <t>Tenants with the My Collections feature enabled need to switch from digest to OAuth.</t>
+    <t>Tenants with the My Collections feature enabled need to switch to OAuth.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Consolidated the dynamic-host ml-config dir into base now that ML 12 is required.
</commit_message>
<xml_diff>
--- a/docs/lux-markdown-tables.xlsx
+++ b/docs/lux-markdown-tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\yale\clones\lux-marklogic-v3\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CE8F3E-107D-4039-8CCC-3ADB654C5248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5E477E6-45F7-4057-B732-24D84A8D212B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="76">
   <si>
     <t>Path</t>
   </si>
@@ -248,12 +248,6 @@
   </si>
   <si>
     <t>[MarkLogic Unit Test user guide](https://marklogic-community.github.io/marklogic-unit-test/)</t>
-  </si>
-  <si>
-    <t>[/dynamic-host](/src/main/ml-config/dynamic-host)</t>
-  </si>
-  <si>
-    <t>Include in all ML 12 deployments, even those that do not require scaling out.  Once we no longer support ML 11, we can merge these settings into the base ml-config dir.</t>
   </si>
   <si>
     <t>[/oauth](/src/main/ml-config/oauth)</t>
@@ -597,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="65.5546875" bestFit="1" customWidth="1"/>
@@ -727,131 +721,123 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D13" t="s">
-        <v>76</v>
+      <c r="C13" t="s">
+        <v>21</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F14" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" t="s">
-        <v>54</v>
+      <c r="D15" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D16" t="s">
-        <v>53</v>
+      <c r="E16" t="s">
+        <v>55</v>
+      </c>
+      <c r="F16" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F18" t="s">
-        <v>49</v>
+        <v>11</v>
+      </c>
+      <c r="G18" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F19" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>61</v>
+      </c>
+      <c r="G20" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F21" t="s">
-        <v>61</v>
-      </c>
-      <c r="G21" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E22" t="s">
-        <v>60</v>
+      <c r="C22" t="s">
+        <v>17</v>
       </c>
       <c r="F22" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" t="s">
-        <v>66</v>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="G23" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="G24" t="s">
-        <v>70</v>
+      <c r="C24" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F25" t="s">
-        <v>69</v>
+        <v>72</v>
+      </c>
+      <c r="G25" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C26" t="s">
-        <v>71</v>
+      <c r="A26" t="s">
+        <v>15</v>
       </c>
       <c r="F26" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>15</v>
-      </c>
-      <c r="F27" t="s">
-        <v>29</v>
-      </c>
-      <c r="G27" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>